<commit_message>
Pooh Points: normal 20260303
</commit_message>
<xml_diff>
--- a/docs/Today_PoohPoints_SEC_ByOwner_2026-03-03.xlsx
+++ b/docs/Today_PoohPoints_SEC_ByOwner_2026-03-03.xlsx
@@ -620,7 +620,7 @@
         <v>1</v>
       </c>
       <c r="P2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q2" t="n">
         <v>5</v>
@@ -674,11 +674,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>4</v>
@@ -690,7 +690,7 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -702,7 +702,7 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q3" t="n">
         <v>2</v>
@@ -838,7 +838,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -866,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q5" t="n">
         <v>1</v>
@@ -920,7 +920,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -948,7 +948,7 @@
         <v>1</v>
       </c>
       <c r="P6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -1233,62 +1233,62 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nijel Pack</t>
+          <t>Denzel Aberdeen</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OU</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>MIZ@OU</t>
+          <t>UK@TA&amp;M</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" t="n">
         <v>12</v>
       </c>
       <c r="Q10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1315,68 +1315,68 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Denzel Aberdeen</t>
+          <t>Nijel Pack</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>OU</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>UK@TA&amp;M</t>
+          <t>MIZ@OU</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H11" t="n">
         <v>6</v>
       </c>
       <c r="I11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P11" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I12" t="n">
         <v>9</v>
@@ -1425,7 +1425,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1440,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Q12" t="n">
         <v>1</v>
@@ -1494,11 +1494,11 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
         <v>3</v>
@@ -1522,19 +1522,19 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q13" t="n">
         <v>1</v>
       </c>
       <c r="R13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S13" t="n">
         <v>1</v>
       </c>
       <c r="T13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1576,14 +1576,14 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1598,13 +1598,13 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="Q14" t="n">
         <v>3</v>
@@ -1619,10 +1619,10 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -1932,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q18" t="n">
         <v>1</v>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -2093,10 +2093,10 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q20" t="n">
         <v>2</v>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -2314,11 +2314,11 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
         <v>2</v>
@@ -2330,7 +2330,7 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23" t="n">
         <v>0</v>
@@ -2342,7 +2342,7 @@
         <v>1</v>
       </c>
       <c r="P23" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q23" t="n">
         <v>1</v>
@@ -2396,7 +2396,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -2482,13 +2482,13 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I25" t="n">
         <v>2</v>
       </c>
       <c r="J25" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -2503,10 +2503,10 @@
         <v>1</v>
       </c>
       <c r="O25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Q25" t="n">
         <v>1</v>
@@ -2560,17 +2560,17 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I26" t="n">
         <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
@@ -2588,13 +2588,13 @@
         <v>1</v>
       </c>
       <c r="P26" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q26" t="n">
         <v>1</v>
       </c>
       <c r="R26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S26" t="n">
         <v>0</v>
@@ -2606,7 +2606,7 @@
         <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -2658,7 +2658,7 @@
         <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -2670,19 +2670,19 @@
         <v>2</v>
       </c>
       <c r="P27" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q27" t="n">
         <v>0</v>
       </c>
       <c r="R27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S27" t="n">
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -2892,10 +2892,10 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I30" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J30" t="n">
         <v>2</v>
@@ -2916,13 +2916,13 @@
         <v>2</v>
       </c>
       <c r="P30" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q30" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R30" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S30" t="n">
         <v>1</v>
@@ -2970,18 +2970,18 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H31" t="n">
+        <v>7</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
         <v>6</v>
       </c>
-      <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="n">
-        <v>5</v>
-      </c>
       <c r="K31" t="n">
         <v>1</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>1</v>
       </c>
       <c r="P31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q31" t="n">
         <v>0</v>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -3138,10 +3138,10 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="I33" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J33" t="n">
         <v>1</v>
@@ -3162,25 +3162,25 @@
         <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -3302,7 +3302,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I35" t="n">
         <v>2</v>
@@ -3311,7 +3311,7 @@
         <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
@@ -3326,7 +3326,7 @@
         <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="Q35" t="n">
         <v>1</v>
@@ -3380,14 +3380,14 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -3408,19 +3408,19 @@
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R36" t="n">
+        <v>6</v>
+      </c>
+      <c r="S36" t="n">
+        <v>2</v>
+      </c>
+      <c r="T36" t="n">
         <v>5</v>
-      </c>
-      <c r="S36" t="n">
-        <v>1</v>
-      </c>
-      <c r="T36" t="n">
-        <v>4</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -3466,7 +3466,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I37" t="n">
         <v>3</v>
@@ -3490,19 +3490,19 @@
         <v>2</v>
       </c>
       <c r="P37" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q37" t="n">
         <v>1</v>
       </c>
       <c r="R37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S37" t="n">
         <v>1</v>
       </c>
       <c r="T37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -3544,7 +3544,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -3651,10 +3651,10 @@
         <v>1</v>
       </c>
       <c r="O39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P39" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q39" t="n">
         <v>1</v>
@@ -3708,11 +3708,11 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I40" t="n">
         <v>14</v>
@@ -3736,19 +3736,19 @@
         <v>0</v>
       </c>
       <c r="P40" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q40" t="n">
         <v>5</v>
       </c>
       <c r="R40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S40" t="n">
         <v>4</v>
       </c>
       <c r="T40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U40" t="n">
         <v>0</v>
@@ -3790,7 +3790,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -3876,13 +3876,13 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I42" t="n">
         <v>20</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -3900,7 +3900,7 @@
         <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q42" t="n">
         <v>8</v>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -4185,62 +4185,62 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kareem Stagg</t>
+          <t>Pop Isaacs</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>UGA</t>
+          <t>TA&amp;M</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>ALA@UGA</t>
+          <t>UK@TA&amp;M</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Halftime</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I46" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M46" t="n">
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O46" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="Q46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -4267,62 +4267,62 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Pop Isaacs</t>
+          <t>Kareem Stagg</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>TA&amp;M</t>
+          <t>UGA</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>UK@TA&amp;M</t>
+          <t>ALA@UGA</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>Halftime</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I47" t="n">
+        <v>10</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
+        <v>2</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2</v>
+      </c>
+      <c r="P47" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q47" t="n">
         <v>4</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="n">
-        <v>4</v>
-      </c>
-      <c r="L47" t="n">
-        <v>2</v>
-      </c>
-      <c r="M47" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" t="n">
-        <v>0</v>
-      </c>
-      <c r="O47" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>2</v>
       </c>
       <c r="R47" t="n">
         <v>5</v>
       </c>
       <c r="S47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U47" t="n">
         <v>0</v>
@@ -4349,32 +4349,32 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EJ Walker</t>
+          <t>Ali Dibba</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TA&amp;M</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>TENN@SC</t>
+          <t>UK@TA&amp;M</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H48" t="n">
+        <v>7</v>
+      </c>
+      <c r="I48" t="n">
         <v>6</v>
       </c>
-      <c r="I48" t="n">
-        <v>5</v>
-      </c>
       <c r="J48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K48" t="n">
         <v>2</v>
@@ -4386,13 +4386,13 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P48" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="Q48" t="n">
         <v>2</v>
@@ -4401,16 +4401,16 @@
         <v>4</v>
       </c>
       <c r="S48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -4431,68 +4431,68 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Jordan Ross</t>
+          <t>EJ Walker</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>UGA</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>ALA@UGA</t>
+          <t>TENN@SC</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Halftime</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H49" t="n">
+        <v>6</v>
+      </c>
+      <c r="I49" t="n">
         <v>5</v>
       </c>
-      <c r="I49" t="n">
-        <v>2</v>
-      </c>
       <c r="J49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K49" t="n">
+        <v>2</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="n">
+        <v>2</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2</v>
+      </c>
+      <c r="P49" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2</v>
+      </c>
+      <c r="R49" t="n">
         <v>4</v>
       </c>
-      <c r="L49" t="n">
-        <v>0</v>
-      </c>
-      <c r="M49" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" t="n">
-        <v>1</v>
-      </c>
-      <c r="O49" t="n">
-        <v>0</v>
-      </c>
-      <c r="P49" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>0</v>
-      </c>
-      <c r="R49" t="n">
-        <v>1</v>
-      </c>
       <c r="S49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T49" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -4513,12 +4513,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>London Jemison</t>
+          <t>Jordan Ross</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>UGA</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4535,34 +4535,34 @@
         <v>5</v>
       </c>
       <c r="I50" t="n">
+        <v>2</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="n">
         <v>4</v>
       </c>
-      <c r="J50" t="n">
-        <v>2</v>
-      </c>
-      <c r="K50" t="n">
-        <v>0</v>
-      </c>
       <c r="L50" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M50" t="n">
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S50" t="n">
         <v>0</v>
@@ -4595,44 +4595,44 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Ali Dibba</t>
+          <t>London Jemison</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TA&amp;M</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>UK@TA&amp;M</t>
+          <t>ALA@UGA</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>Halftime</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I51" t="n">
         <v>4</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M51" t="n">
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O51" t="n">
         <v>1</v>
@@ -4644,13 +4644,13 @@
         <v>1</v>
       </c>
       <c r="R51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S51" t="n">
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U51" t="n">
         <v>2</v>
@@ -4677,68 +4677,68 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Bishop Boswell</t>
+          <t>T.O. Barrett</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TENN</t>
+          <t>MIZ</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>TENN@SC</t>
+          <t>MIZ@OU</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H52" t="n">
+        <v>5</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1</v>
+      </c>
+      <c r="L52" t="n">
+        <v>1</v>
+      </c>
+      <c r="M52" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" t="n">
+        <v>2</v>
+      </c>
+      <c r="P52" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>1</v>
+      </c>
+      <c r="R52" t="n">
         <v>4</v>
       </c>
-      <c r="I52" t="n">
-        <v>6</v>
-      </c>
-      <c r="J52" t="n">
-        <v>3</v>
-      </c>
-      <c r="K52" t="n">
-        <v>2</v>
-      </c>
-      <c r="L52" t="n">
-        <v>1</v>
-      </c>
-      <c r="M52" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" t="n">
-        <v>2</v>
-      </c>
-      <c r="O52" t="n">
-        <v>3</v>
-      </c>
-      <c r="P52" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>2</v>
-      </c>
-      <c r="R52" t="n">
-        <v>8</v>
-      </c>
       <c r="S52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V52" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -4759,22 +4759,22 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Brandon Garrison</t>
+          <t>Bishop Boswell</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>TENN</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>UK@TA&amp;M</t>
+          <t>TENN@SC</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H53" t="n">
@@ -4784,10 +4784,10 @@
         <v>6</v>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4799,22 +4799,22 @@
         <v>2</v>
       </c>
       <c r="O53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P53" t="n">
+        <v>29</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>2</v>
+      </c>
+      <c r="R53" t="n">
         <v>8</v>
       </c>
-      <c r="Q53" t="n">
-        <v>3</v>
-      </c>
-      <c r="R53" t="n">
+      <c r="S53" t="n">
+        <v>2</v>
+      </c>
+      <c r="T53" t="n">
         <v>4</v>
-      </c>
-      <c r="S53" t="n">
-        <v>0</v>
-      </c>
-      <c r="T53" t="n">
-        <v>1</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -4841,53 +4841,53 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>T.O. Barrett</t>
+          <t>Brandon Garrison</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MIZ</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>MIZ@OU</t>
+          <t>UK@TA&amp;M</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H54" t="n">
         <v>4</v>
       </c>
       <c r="I54" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J54" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O54" t="n">
         <v>1</v>
       </c>
       <c r="P54" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="Q54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R54" t="n">
         <v>4</v>
@@ -4899,10 +4899,10 @@
         <v>1</v>
       </c>
       <c r="U54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V54" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H55" t="n">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H56" t="n">
@@ -5102,7 +5102,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H58" t="n">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H60" t="n">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H62" t="n">
@@ -5540,7 +5540,7 @@
         <v>0</v>
       </c>
       <c r="P62" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q62" t="n">
         <v>1</v>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H65" t="n">
@@ -5786,7 +5786,7 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q65" t="n">
         <v>0</v>
@@ -5840,7 +5840,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H66" t="n">
@@ -5907,22 +5907,22 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Dayton Forsythe</t>
+          <t>Jake Wilkins</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OU</t>
+          <t>UGA</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>MIZ@OU</t>
+          <t>ALA@UGA</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>Halftime</t>
         </is>
       </c>
       <c r="H67" t="n">
@@ -5935,7 +5935,7 @@
         <v>1</v>
       </c>
       <c r="K67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L67" t="n">
         <v>0</v>
@@ -5944,13 +5944,13 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P67" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q67" t="n">
         <v>0</v>
@@ -5962,7 +5962,7 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -5989,29 +5989,29 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Jake Wilkins</t>
+          <t>Jordan Butler</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>UGA</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>ALA@UGA</t>
+          <t>TENN@SC</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Halftime</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H68" t="n">
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J68" t="n">
         <v>1</v>
@@ -6029,16 +6029,16 @@
         <v>0</v>
       </c>
       <c r="O68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P68" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="Q68" t="n">
         <v>0</v>
       </c>
       <c r="R68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S68" t="n">
         <v>0</v>
@@ -6047,10 +6047,10 @@
         <v>1</v>
       </c>
       <c r="U68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69">
@@ -6071,32 +6071,32 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Jordan Butler</t>
+          <t>Justin Bailey</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>UGA</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>TENN@SC</t>
+          <t>ALA@UGA</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Halftime</t>
         </is>
       </c>
       <c r="H69" t="n">
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -6111,28 +6111,28 @@
         <v>0</v>
       </c>
       <c r="O69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P69" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="Q69" t="n">
         <v>0</v>
       </c>
       <c r="R69" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S69" t="n">
         <v>0</v>
       </c>
       <c r="T69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -6153,22 +6153,22 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Justin Bailey</t>
+          <t>Trent Noah</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>UGA</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>ALA@UGA</t>
+          <t>UK@TA&amp;M</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Halftime</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H70" t="n">
@@ -6178,7 +6178,7 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -6193,22 +6193,22 @@
         <v>0</v>
       </c>
       <c r="O70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P70" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q70" t="n">
         <v>0</v>
       </c>
       <c r="R70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S70" t="n">
         <v>0</v>
       </c>
       <c r="T70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U70" t="n">
         <v>0</v>
@@ -6235,12 +6235,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Trent Noah</t>
+          <t>Zach Clemence</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>TA&amp;M</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -6250,17 +6250,17 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:20 - 1st Half</t>
         </is>
       </c>
       <c r="H71" t="n">
         <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -6275,7 +6275,7 @@
         <v>0</v>
       </c>
       <c r="O71" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P71" t="n">
         <v>7</v>
@@ -6284,7 +6284,7 @@
         <v>0</v>
       </c>
       <c r="R71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S71" t="n">
         <v>0</v>
@@ -6293,10 +6293,10 @@
         <v>2</v>
       </c>
       <c r="U71" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V71" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -6317,35 +6317,35 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Zach Clemence</t>
+          <t>Dayton Forsythe</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TA&amp;M</t>
+          <t>OU</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>UK@TA&amp;M</t>
+          <t>MIZ@OU</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>4:57 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J72" t="n">
         <v>1</v>
       </c>
       <c r="K72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" t="n">
         <v>0</v>
@@ -6354,31 +6354,31 @@
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P72" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q72" t="n">
         <v>0</v>
       </c>
       <c r="R72" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S72" t="n">
         <v>0</v>
       </c>
       <c r="T72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H73" t="n">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>0:49 - 2nd Half</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="H75" t="n">
@@ -6660,7 +6660,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>5:01 - 1st Half</t>
+          <t>3:31 - 1st Half</t>
         </is>
       </c>
       <c r="H76" t="n">
@@ -6761,27 +6761,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hilton Heads</t>
+          <t>G-Flop</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>G-Flop</t>
+          <t>Hilton Heads</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -6817,7 +6817,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" t="n">
         <v>3</v>
@@ -6830,7 +6830,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" t="n">
         <v>3</v>

</xml_diff>